<commit_message>
update exel cooperation aggreement
</commit_message>
<xml_diff>
--- a/resources/templates/exel_cooperation_agreement-bulk-template.xlsx
+++ b/resources/templates/exel_cooperation_agreement-bulk-template.xlsx
@@ -470,10 +470,10 @@
         <v>operationalCostAllowanceUnit</v>
       </c>
       <c r="X1" t="str">
-        <v>tlAllowance</v>
+        <v>jabatanAllowance</v>
       </c>
       <c r="Y1" t="str">
-        <v>tlAllowanceUnit</v>
+        <v>jabatanAllowanceUnit</v>
       </c>
       <c r="Z1" t="str">
         <v>partnerBankAccountNumber</v>

</xml_diff>